<commit_message>
Update Book1.xlsx and add Details.xlsx sample data
</commit_message>
<xml_diff>
--- a/EXCEL/Book1.xlsx
+++ b/EXCEL/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{12CB6B68-B445-4F67-9E16-1EDCB2507310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{323593B7-15A6-4D03-B713-38800297BFF8}"/>
+  <xr:revisionPtr revIDLastSave="99" documentId="13_ncr:1_{12CB6B68-B445-4F67-9E16-1EDCB2507310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59F297B4-E546-481D-B3A9-32A409B45508}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{74739673-5005-4586-AACD-5642EFA35219}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
   <si>
     <t>SUNDAY</t>
   </si>
@@ -124,13 +124,43 @@
   </si>
   <si>
     <t>result</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">salary </t>
+  </si>
+  <si>
+    <t>new salary</t>
+  </si>
+  <si>
+    <t>dhruv</t>
+  </si>
+  <si>
+    <t>darsh</t>
+  </si>
+  <si>
+    <t>dhruvi</t>
+  </si>
+  <si>
+    <t>hike</t>
+  </si>
+  <si>
+    <t>relative refrencing</t>
+  </si>
+  <si>
+    <t>mixed ref</t>
+  </si>
+  <si>
+    <t>absolute</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,13 +174,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -165,8 +208,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -505,10 +552,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6598AFA-676A-4076-87A0-8BC075595178}">
-  <dimension ref="B3:Q29"/>
+  <dimension ref="B3:Q33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -698,7 +746,10 @@
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
       <c r="J17">
         <v>10002</v>
       </c>
@@ -706,7 +757,16 @@
         <v>124</v>
       </c>
     </row>
-    <row r="18" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" t="s">
+        <v>24</v>
+      </c>
       <c r="J18">
         <v>10002</v>
       </c>
@@ -714,7 +774,17 @@
         <v>125</v>
       </c>
     </row>
-    <row r="19" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C19">
+        <v>50000</v>
+      </c>
+      <c r="D19" s="2">
+        <f>C19+(C19*$C$23)</f>
+        <v>65000</v>
+      </c>
       <c r="J19">
         <v>10002</v>
       </c>
@@ -722,7 +792,17 @@
         <v>126</v>
       </c>
     </row>
-    <row r="20" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20">
+        <v>42000</v>
+      </c>
+      <c r="D20" s="2">
+        <f t="shared" ref="D20:D21" si="0">C20+(C20*$C$23)</f>
+        <v>54600</v>
+      </c>
       <c r="J20">
         <v>10002</v>
       </c>
@@ -733,7 +813,17 @@
         <v>555</v>
       </c>
     </row>
-    <row r="21" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21">
+        <v>63000</v>
+      </c>
+      <c r="D21" s="2">
+        <f t="shared" si="0"/>
+        <v>81900</v>
+      </c>
       <c r="J21">
         <v>10002</v>
       </c>
@@ -744,7 +834,8 @@
         <v>556</v>
       </c>
     </row>
-    <row r="22" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="D22" s="1"/>
       <c r="J22">
         <v>10002</v>
       </c>
@@ -755,7 +846,13 @@
         <v>557</v>
       </c>
     </row>
-    <row r="23" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0.3</v>
+      </c>
       <c r="J23">
         <v>10002</v>
       </c>
@@ -763,7 +860,13 @@
         <v>558</v>
       </c>
     </row>
-    <row r="24" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B24" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
       <c r="J24">
         <v>10002</v>
       </c>
@@ -771,7 +874,19 @@
         <v>559</v>
       </c>
     </row>
-    <row r="25" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B25" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0.1</v>
+      </c>
       <c r="J25">
         <v>10002</v>
       </c>
@@ -779,7 +894,21 @@
         <v>560</v>
       </c>
     </row>
-    <row r="26" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B26" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="3">
+        <v>50000</v>
+      </c>
+      <c r="D26" s="3">
+        <f>$C26*D$25</f>
+        <v>2500</v>
+      </c>
+      <c r="E26" s="3">
+        <f>$C26*E$25</f>
+        <v>5000</v>
+      </c>
       <c r="J26">
         <v>10002</v>
       </c>
@@ -787,7 +916,21 @@
         <v>561</v>
       </c>
     </row>
-    <row r="27" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B27" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="3">
+        <v>42000</v>
+      </c>
+      <c r="D27" s="3">
+        <f t="shared" ref="D27:E28" si="1">$C27*D$25</f>
+        <v>2100</v>
+      </c>
+      <c r="E27" s="3">
+        <f t="shared" si="1"/>
+        <v>4200</v>
+      </c>
       <c r="J27">
         <v>10002</v>
       </c>
@@ -795,7 +938,21 @@
         <v>562</v>
       </c>
     </row>
-    <row r="28" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B28" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="3">
+        <v>63000</v>
+      </c>
+      <c r="D28" s="3">
+        <f t="shared" si="1"/>
+        <v>3150</v>
+      </c>
+      <c r="E28" s="3">
+        <f t="shared" si="1"/>
+        <v>6300</v>
+      </c>
       <c r="J28">
         <v>10002</v>
       </c>
@@ -803,9 +960,52 @@
         <v>563</v>
       </c>
     </row>
-    <row r="29" spans="10:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:14" x14ac:dyDescent="0.3">
       <c r="N29">
         <v>564</v>
+      </c>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B32">
+        <v>25</v>
+      </c>
+      <c r="C32">
+        <v>36</v>
+      </c>
+      <c r="D32">
+        <f>B32+C32</f>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B33">
+        <v>56</v>
+      </c>
+      <c r="C33">
+        <v>54</v>
+      </c>
+      <c r="D33" cm="1">
+        <f t="array" ref="D33:E33">B33:C33</f>
+        <v>56</v>
+      </c>
+      <c r="E33">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>